<commit_message>
21/09/2026 update (manuscript results)
</commit_message>
<xml_diff>
--- a/Figures_source_data/Figure 4.xlsx
+++ b/Figures_source_data/Figure 4.xlsx
@@ -1216,31 +1216,31 @@
         <v>9</v>
       </c>
       <c r="B3" s="9">
-        <v>52.9050899654778</v>
+        <v>52.5444881438454</v>
       </c>
       <c r="C3" s="9">
-        <v>33.7913127334939</v>
+        <v>33.708507382722</v>
       </c>
       <c r="D3" s="9">
         <v>216.107744877251</v>
       </c>
       <c r="E3" s="9">
-        <v>32.9355063087086</v>
+        <v>32.9509362744001</v>
       </c>
       <c r="F3" s="9">
-        <v>335.739653884932</v>
+        <v>335.311676678219</v>
       </c>
       <c r="G3" s="9">
-        <v>64.8996198367579</v>
+        <v>64.8970151674558</v>
       </c>
       <c r="H3" s="9">
         <v>9.91966703850433</v>
       </c>
       <c r="I3" s="9">
-        <v>62.5747188931541</v>
+        <v>62.6414063051297</v>
       </c>
       <c r="J3" s="10">
-        <v>137.394005768416</v>
+        <v>137.45808851109</v>
       </c>
     </row>
     <row r="4" ht="15" spans="1:10">
@@ -1248,31 +1248,31 @@
         <v>10</v>
       </c>
       <c r="B4" s="9">
-        <v>52.9050899654778</v>
+        <v>52.5444881438454</v>
       </c>
       <c r="C4" s="9">
-        <v>33.7913127334939</v>
+        <v>33.708507382722</v>
       </c>
       <c r="D4" s="9">
         <v>216.107744877251</v>
       </c>
       <c r="E4" s="9">
-        <v>32.9355063087086</v>
+        <v>32.9509362744001</v>
       </c>
       <c r="F4" s="9">
-        <v>335.739653884932</v>
+        <v>335.311676678219</v>
       </c>
       <c r="G4" s="9">
-        <v>64.8996198367579</v>
+        <v>64.8970151674558</v>
       </c>
       <c r="H4" s="9">
         <v>9.91966703850433</v>
       </c>
       <c r="I4" s="9">
-        <v>62.5747188931541</v>
+        <v>62.6414063051297</v>
       </c>
       <c r="J4" s="10">
-        <v>137.394005768416</v>
+        <v>137.45808851109</v>
       </c>
     </row>
     <row r="5" ht="15" spans="1:10">
@@ -1280,31 +1280,31 @@
         <v>11</v>
       </c>
       <c r="B5" s="12">
-        <v>52.9050899654778</v>
+        <v>52.5444881438454</v>
       </c>
       <c r="C5" s="12">
-        <v>33.7913127334939</v>
+        <v>33.708507382722</v>
       </c>
       <c r="D5" s="12">
         <v>216.107744877251</v>
       </c>
       <c r="E5" s="12">
-        <v>32.9355063087086</v>
+        <v>32.9509362744001</v>
       </c>
       <c r="F5" s="12">
-        <v>335.739653884932</v>
+        <v>335.311676678219</v>
       </c>
       <c r="G5" s="12">
-        <v>64.8996198367579</v>
+        <v>64.8970151674558</v>
       </c>
       <c r="H5" s="12">
         <v>9.91966703850433</v>
       </c>
       <c r="I5" s="12">
-        <v>62.5747188931541</v>
+        <v>62.6414063051297</v>
       </c>
       <c r="J5" s="13">
-        <v>137.394005768416</v>
+        <v>137.45808851109</v>
       </c>
     </row>
     <row r="6" ht="15" spans="1:10">
@@ -1368,7 +1368,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="9">
-        <v>65.1603529116776</v>
+        <v>64.689398990779</v>
       </c>
       <c r="C9" s="9">
         <v>40.1806775258352</v>
@@ -1377,22 +1377,22 @@
         <v>218.561635265672</v>
       </c>
       <c r="E9" s="9">
-        <v>34.2588324623488</v>
+        <v>34.2779512338034</v>
       </c>
       <c r="F9" s="9">
-        <v>358.161498165531</v>
+        <v>357.70966301609</v>
       </c>
       <c r="G9" s="9">
-        <v>80.7164319113492</v>
+        <v>80.7349969665225</v>
       </c>
       <c r="H9" s="9">
         <v>9.57035186038771</v>
       </c>
       <c r="I9" s="9">
-        <v>65.9149165079445</v>
+        <v>65.9972281481682</v>
       </c>
       <c r="J9" s="10">
-        <v>156.201700279681</v>
+        <v>156.302576975079</v>
       </c>
     </row>
     <row r="10" ht="15" spans="1:10">
@@ -1400,7 +1400,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="9">
-        <v>67.5505380247698</v>
+        <v>67.0569545465475</v>
       </c>
       <c r="C10" s="9">
         <v>41.2915077606034</v>
@@ -1409,22 +1409,22 @@
         <v>210.112694393926</v>
       </c>
       <c r="E10" s="9">
-        <v>32.7745749765467</v>
+        <v>32.794801704182</v>
       </c>
       <c r="F10" s="9">
-        <v>351.729315155844</v>
+        <v>351.255958405261</v>
       </c>
       <c r="G10" s="9">
-        <v>82.0813233078892</v>
+        <v>82.0963327181375</v>
       </c>
       <c r="H10" s="9">
         <v>9.14575501202569</v>
       </c>
       <c r="I10" s="9">
-        <v>64.2868817578727</v>
+        <v>64.3731896554867</v>
       </c>
       <c r="J10" s="10">
-        <v>155.513960077787</v>
+        <v>155.615277385649</v>
       </c>
     </row>
     <row r="11" ht="15" spans="1:10">
@@ -1432,7 +1432,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="9">
-        <v>67.4740261463381</v>
+        <v>66.9857638775213</v>
       </c>
       <c r="C11" s="9">
         <v>42.1196224367412</v>
@@ -1441,22 +1441,22 @@
         <v>207.976509525362</v>
       </c>
       <c r="E11" s="9">
-        <v>36.8275381902722</v>
+        <v>36.8472495336702</v>
       </c>
       <c r="F11" s="9">
-        <v>354.397696298714</v>
+        <v>353.929145373299</v>
       </c>
       <c r="G11" s="9">
-        <v>83.6837723742932</v>
+        <v>83.7080520660971</v>
       </c>
       <c r="H11" s="9">
         <v>9.06493178368252</v>
       </c>
       <c r="I11" s="9">
-        <v>66.44514938815</v>
+        <v>66.529515283961</v>
       </c>
       <c r="J11" s="10">
-        <v>159.193853546126</v>
+        <v>159.302499133738</v>
       </c>
     </row>
     <row r="12" ht="15" spans="1:10">
@@ -1464,7 +1464,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="9">
-        <v>109.391550568324</v>
+        <v>108.61794768786</v>
       </c>
       <c r="C12" s="9">
         <v>53.3283273946571</v>
@@ -1473,22 +1473,22 @@
         <v>155.864194312196</v>
       </c>
       <c r="E12" s="9">
-        <v>26.7435526119989</v>
+        <v>26.7749407330556</v>
       </c>
       <c r="F12" s="9">
-        <v>345.327624887175</v>
+        <v>344.585410127768</v>
       </c>
       <c r="G12" s="9">
-        <v>113.177594426998</v>
+        <v>113.189507288193</v>
       </c>
       <c r="H12" s="9">
         <v>6.84662112996961</v>
       </c>
       <c r="I12" s="9">
-        <v>58.8633304764823</v>
+        <v>58.9882445591715</v>
       </c>
       <c r="J12" s="10">
-        <v>178.887546033449</v>
+        <v>179.024372977334</v>
       </c>
     </row>
     <row r="13" ht="15" spans="1:10">
@@ -1496,7 +1496,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="9">
-        <v>28.9154721991423</v>
+        <v>28.8270576185802</v>
       </c>
       <c r="C13" s="9">
         <v>40.1806775258352</v>
@@ -1505,22 +1505,22 @@
         <v>218.561635265672</v>
       </c>
       <c r="E13" s="9">
-        <v>34.2588324623488</v>
+        <v>34.2779512338034</v>
       </c>
       <c r="F13" s="9">
-        <v>321.916617452998</v>
+        <v>321.847321643889</v>
       </c>
       <c r="G13" s="9">
-        <v>32.2865727645399</v>
+        <v>32.2939987866083</v>
       </c>
       <c r="H13" s="9">
         <v>9.57035186038771</v>
       </c>
       <c r="I13" s="9">
-        <v>65.9149165079445</v>
+        <v>65.9972281481682</v>
       </c>
       <c r="J13" s="10">
-        <v>107.771841132872</v>
+        <v>107.861578795165</v>
       </c>
     </row>
     <row r="14" ht="15" spans="1:10">
@@ -1528,7 +1528,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="12">
-        <v>46.7478931141162</v>
+        <v>46.5617253409708</v>
       </c>
       <c r="C14" s="12">
         <v>53.3283273946571</v>
@@ -1537,22 +1537,22 @@
         <v>155.864194312196</v>
       </c>
       <c r="E14" s="12">
-        <v>26.7435526119989</v>
+        <v>26.7749407330556</v>
       </c>
       <c r="F14" s="12">
-        <v>282.683967432965</v>
+        <v>282.52918778088</v>
       </c>
       <c r="G14" s="12">
-        <v>45.2710377707994</v>
+        <v>45.2758029152771</v>
       </c>
       <c r="H14" s="12">
         <v>6.84662112996961</v>
       </c>
       <c r="I14" s="12">
-        <v>58.8633304764823</v>
+        <v>58.9882445591715</v>
       </c>
       <c r="J14" s="13">
-        <v>110.98098937725</v>
+        <v>111.110668604418</v>
       </c>
     </row>
     <row r="15" ht="15" spans="1:10">
@@ -1616,7 +1616,7 @@
         <v>9</v>
       </c>
       <c r="B18" s="9">
-        <v>79.6451993295904</v>
+        <v>79.0295827395075</v>
       </c>
       <c r="C18" s="9">
         <v>47.5737182842934</v>
@@ -1625,22 +1625,22 @@
         <v>216.817462046977</v>
       </c>
       <c r="E18" s="9">
-        <v>38.8316319796722</v>
+        <v>38.8560216638447</v>
       </c>
       <c r="F18" s="9">
-        <v>382.868011640534</v>
+        <v>382.27678473462</v>
       </c>
       <c r="G18" s="9">
-        <v>90.6465815299092</v>
+        <v>90.6536488514867</v>
       </c>
       <c r="H18" s="9">
         <v>8.80382172475935</v>
       </c>
       <c r="I18" s="9">
-        <v>74.3374820317466</v>
+        <v>74.4399580351931</v>
       </c>
       <c r="J18" s="10">
-        <v>173.787885286414</v>
+        <v>173.897428611438</v>
       </c>
     </row>
     <row r="19" ht="15" spans="1:10">
@@ -1648,7 +1648,7 @@
         <v>10</v>
       </c>
       <c r="B19" s="9">
-        <v>90.4650368826121</v>
+        <v>89.7616110005325</v>
       </c>
       <c r="C19" s="9">
         <v>50.9269005591324</v>
@@ -1657,22 +1657,22 @@
         <v>193.663668391264</v>
       </c>
       <c r="E19" s="9">
-        <v>34.3064876321572</v>
+        <v>34.3352223324636</v>
       </c>
       <c r="F19" s="9">
-        <v>369.362093465164</v>
+        <v>368.687402283392</v>
       </c>
       <c r="G19" s="9">
-        <v>97.1475895496584</v>
+        <v>97.1387051277554</v>
       </c>
       <c r="H19" s="9">
         <v>7.64656664411865</v>
       </c>
       <c r="I19" s="9">
-        <v>71.469422622912</v>
+        <v>71.5871683961445</v>
       </c>
       <c r="J19" s="10">
-        <v>176.263578816688</v>
+        <v>176.372440168018</v>
       </c>
     </row>
     <row r="20" ht="15" spans="1:10">
@@ -1680,7 +1680,7 @@
         <v>11</v>
       </c>
       <c r="B20" s="12">
-        <v>89.5619252471207</v>
+        <v>88.8510673733556</v>
       </c>
       <c r="C20" s="12">
         <v>53.1871412430887</v>
@@ -1689,22 +1689,22 @@
         <v>184.910455346435</v>
       </c>
       <c r="E20" s="12">
-        <v>43.028534605048</v>
+        <v>43.0549983852771</v>
       </c>
       <c r="F20" s="12">
-        <v>370.688056441692</v>
+        <v>370.003662348154</v>
       </c>
       <c r="G20" s="12">
-        <v>98.758785746557</v>
+        <v>98.7766386406</v>
       </c>
       <c r="H20" s="12">
         <v>7.36850344107293</v>
       </c>
       <c r="I20" s="12">
-        <v>75.9487936607636</v>
+        <v>76.0581011247921</v>
       </c>
       <c r="J20" s="13">
-        <v>182.076082848392</v>
+        <v>182.203243206466</v>
       </c>
     </row>
     <row r="21" ht="15" spans="1:10">
@@ -1768,7 +1768,7 @@
         <v>9</v>
       </c>
       <c r="B24" s="9">
-        <v>96.7988363062516</v>
+        <v>96.0212741284477</v>
       </c>
       <c r="C24" s="9">
         <v>54.7846759387106</v>
@@ -1777,22 +1777,22 @@
         <v>191.664922687602</v>
       </c>
       <c r="E24" s="9">
-        <v>41.4867358643995</v>
+        <v>41.5169031081362</v>
       </c>
       <c r="F24" s="9">
-        <v>384.735170796967</v>
+        <v>383.9877758629</v>
       </c>
       <c r="G24" s="9">
-        <v>101.107747981998</v>
+        <v>101.102324553008</v>
       </c>
       <c r="H24" s="9">
         <v>7.96757577389465</v>
       </c>
       <c r="I24" s="9">
-        <v>72.9378933174645</v>
+        <v>73.0613208799764</v>
       </c>
       <c r="J24" s="10">
-        <v>182.013217073359</v>
+        <v>182.13122120688</v>
       </c>
     </row>
     <row r="25" ht="15" spans="1:10">
@@ -1800,7 +1800,7 @@
         <v>10</v>
       </c>
       <c r="B25" s="9">
-        <v>116.698671288556</v>
+        <v>115.782115427429</v>
       </c>
       <c r="C25" s="9">
         <v>59.2893688882769</v>
@@ -1809,22 +1809,22 @@
         <v>149.691290648084</v>
       </c>
       <c r="E25" s="9">
-        <v>32.2986994719699</v>
+        <v>32.3371931809708</v>
       </c>
       <c r="F25" s="9">
-        <v>357.97803029689</v>
+        <v>357.099968144759</v>
       </c>
       <c r="G25" s="9">
-        <v>113.751415962957</v>
+        <v>113.725305120345</v>
       </c>
       <c r="H25" s="9">
         <v>6.34514022387964</v>
       </c>
       <c r="I25" s="9">
-        <v>64.8210551760345</v>
+        <v>64.9722746961923</v>
       </c>
       <c r="J25" s="10">
-        <v>184.91761136287</v>
+        <v>185.042720040417</v>
       </c>
     </row>
     <row r="26" ht="15" spans="1:10">
@@ -1832,7 +1832,7 @@
         <v>11</v>
       </c>
       <c r="B26" s="9">
-        <v>118.517413020325</v>
+        <v>117.515909191184</v>
       </c>
       <c r="C26" s="9">
         <v>62.6545259434911</v>
@@ -1841,22 +1841,22 @@
         <v>132.658623393498</v>
       </c>
       <c r="E26" s="9">
-        <v>41.7321530939241</v>
+        <v>41.7670349196341</v>
       </c>
       <c r="F26" s="9">
-        <v>355.562715451241</v>
+        <v>354.596093447805</v>
       </c>
       <c r="G26" s="9">
-        <v>118.059931201959</v>
+        <v>118.072847885318</v>
       </c>
       <c r="H26" s="9">
         <v>5.86914443184781</v>
       </c>
       <c r="I26" s="9">
-        <v>68.5695007503177</v>
+        <v>68.7086217063099</v>
       </c>
       <c r="J26" s="10">
-        <v>192.49857638412</v>
+        <v>192.650614023475</v>
       </c>
     </row>
     <row r="27" ht="15" spans="1:10">

</xml_diff>